<commit_message>
paper run 2026-10-26 09:34
</commit_message>
<xml_diff>
--- a/reports/2026-10-26.xlsx
+++ b/reports/2026-10-26.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,135 @@
       </c>
       <c r="K4" t="n">
         <v>21.62</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-26T07:11:58.291394+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8.68</v>
+      </c>
+      <c r="G5" t="n">
+        <v>14</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00158</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>5.32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-26T07:41:35.590545+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F6" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="G6" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00108</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>10.81</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-26T09:23:46.232294+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.00159</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>2.52</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -646,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -676,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37.37</v>
+        <v>56.02</v>
       </c>
     </row>
     <row r="7">
@@ -686,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>37.37</v>
+        <v>56.02</v>
       </c>
     </row>
     <row r="8">
@@ -716,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4186.799999999999</v>
+        <v>4205.45</v>
       </c>
     </row>
     <row r="12">
@@ -767,16 +896,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>-261.66</v>
+        <v>134.06</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>21.13</v>
       </c>
     </row>
     <row r="16">
@@ -786,16 +915,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>726.99</v>
+        <v>871.0700000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>32.37</v>
+        <v>34.89</v>
       </c>
     </row>
     <row r="17">
@@ -812,16 +941,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>165.71</v>
+        <v>445.08</v>
       </c>
       <c r="E18" t="n">
-        <v>32.37</v>
+        <v>43.18</v>
       </c>
     </row>
     <row r="19">
@@ -831,16 +960,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>317.45</v>
+        <v>433.8</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>10.32</v>
       </c>
     </row>
     <row r="20">
@@ -850,16 +979,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>-17.83</v>
+        <v>126.25</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="21">
@@ -876,16 +1005,16 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" t="n">
         <v>4</v>
       </c>
-      <c r="C22" t="n">
-        <v>3</v>
-      </c>
       <c r="D22" t="n">
-        <v>364.25</v>
+        <v>542.0700000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>21.62</v>
+        <v>32.43</v>
       </c>
     </row>
     <row r="23">
@@ -895,16 +1024,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>153.4</v>
+        <v>297.48</v>
       </c>
       <c r="E23" t="n">
-        <v>10.75</v>
+        <v>13.27</v>
       </c>
     </row>
     <row r="24">
@@ -914,16 +1043,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>-52.32</v>
+        <v>165.58</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>10.32</v>
       </c>
     </row>
     <row r="25">
@@ -940,13 +1069,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>27.34</v>
+        <v>128.89</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -959,16 +1088,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>437.99</v>
+        <v>876.24</v>
       </c>
       <c r="E27" t="n">
-        <v>37.37</v>
+        <v>56.02</v>
       </c>
     </row>
     <row r="29">
@@ -1007,13 +1136,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>32.37</v>
+        <v>43.18</v>
       </c>
     </row>
     <row r="33">
@@ -1023,111 +1152,111 @@
         </is>
       </c>
       <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>10.32</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
         <v>1</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C34" t="n">
         <v>1</v>
       </c>
-      <c r="D33" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="D34" t="n">
+        <v>2.52</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>5</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>21.13</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>2</v>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" t="n">
-        <v>32.37</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>34.89</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>10.75</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1137,13 +1266,13 @@
         <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>10.75</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1153,35 +1282,45 @@
         <v>1</v>
       </c>
       <c r="D42" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
         <v>21.62</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>16.13</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1191,121 +1330,121 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>21.62</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
-        <v>10.75</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
-        <v>5</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>32.43</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="n">
+        <v>13.27</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" t="n">
-        <v>21.62</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="n">
-        <v>15.75</v>
+        <v>10.32</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="n">
+        <v>32.43</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1315,23 +1454,77 @@
         <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>32.37</v>
+        <v>15.75</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>7.84</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" t="n">
+        <v>40.21</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B55" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
-        <v>5</v>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="n">
+        <v>15.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-26 18:03
</commit_message>
<xml_diff>
--- a/reports/2026-10-26.xlsx
+++ b/reports/2026-10-26.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -730,6 +730,49 @@
       </c>
       <c r="K7" t="n">
         <v>2.52</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-26T14:04:22.153866+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>29</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.00129</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>11.6</v>
       </c>
     </row>
   </sheetData>
@@ -743,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -765,7 +808,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -775,7 +818,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -805,7 +848,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56.02</v>
+        <v>67.62</v>
       </c>
     </row>
     <row r="7">
@@ -815,7 +858,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>56.02</v>
+        <v>67.62</v>
       </c>
     </row>
     <row r="8">
@@ -845,7 +888,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4205.45</v>
+        <v>4217.05</v>
       </c>
     </row>
     <row r="12">
@@ -896,13 +939,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>134.06</v>
+        <v>290.83</v>
       </c>
       <c r="E15" t="n">
         <v>21.13</v>
@@ -915,16 +958,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>871.0700000000001</v>
+        <v>1424.14</v>
       </c>
       <c r="E16" t="n">
-        <v>34.89</v>
+        <v>46.49</v>
       </c>
     </row>
     <row r="17">
@@ -937,288 +980,291 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>445.08</v>
+        <v>202.03</v>
       </c>
       <c r="E18" t="n">
-        <v>43.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>433.8</v>
+        <v>445.08</v>
       </c>
       <c r="E19" t="n">
-        <v>10.32</v>
+        <v>43.18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>126.25</v>
+        <v>784.84</v>
       </c>
       <c r="E20" t="n">
-        <v>2.52</v>
+        <v>21.92</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>283.02</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.52</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>5</v>
-      </c>
-      <c r="C22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" t="n">
-        <v>542.0700000000001</v>
-      </c>
-      <c r="E22" t="n">
-        <v>32.43</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>297.48</v>
+        <v>954.96</v>
       </c>
       <c r="E23" t="n">
-        <v>13.27</v>
+        <v>32.43</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>165.58</v>
+        <v>594.4299999999999</v>
       </c>
       <c r="E24" t="n">
-        <v>10.32</v>
+        <v>24.87</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>165.58</v>
+      </c>
+      <c r="E25" t="n">
+        <v>10.32</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>5</v>
-      </c>
-      <c r="C26" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" t="n">
-        <v>128.89</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NO_LIQUIDITY</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
         <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>876.24</v>
+        <v>698.55</v>
       </c>
       <c r="E27" t="n">
-        <v>56.02</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1016.42</v>
+      </c>
+      <c r="E28" t="n">
+        <v>67.62</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>3</v>
-      </c>
-      <c r="C32" t="n">
-        <v>3</v>
-      </c>
-      <c r="D32" t="n">
-        <v>43.18</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>10.32</v>
+        <v>43.18</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>21.92</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>XRP</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B35" t="n">
         <v>1</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C35" t="n">
         <v>1</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>2.52</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>3</v>
-      </c>
-      <c r="C37" t="n">
-        <v>3</v>
-      </c>
-      <c r="D37" t="n">
-        <v>21.13</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1228,51 +1274,51 @@
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>34.89</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>21.13</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>46.49</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>10.75</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1282,13 +1328,13 @@
         <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>10.75</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1298,99 +1344,99 @@
         <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>21.62</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>16.13</v>
+        <v>21.62</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
+        <v>16.13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B46" t="n">
         <v>1</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C46" t="n">
         <v>1</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>2.52</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>2</v>
-      </c>
-      <c r="C48" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" t="n">
-        <v>32.43</v>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>11.6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>2</v>
-      </c>
-      <c r="C49" t="n">
-        <v>2</v>
-      </c>
-      <c r="D49" t="n">
-        <v>13.27</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1400,67 +1446,67 @@
         <v>2</v>
       </c>
       <c r="D50" t="n">
-        <v>10.32</v>
+        <v>32.43</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>24.87</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
         <v>2</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C52" t="n">
         <v>2</v>
       </c>
-      <c r="D53" t="n">
-        <v>32.43</v>
+      <c r="D52" t="n">
+        <v>10.32</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="n">
-        <v>15.75</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1470,60 +1516,92 @@
         <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>7.84</v>
+        <v>32.43</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>27.35</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>4</v>
-      </c>
-      <c r="C58" t="n">
-        <v>4</v>
-      </c>
-      <c r="D58" t="n">
-        <v>40.21</v>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>7.84</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="n">
+        <v>51.81</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="B61" t="n">
         <v>2</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C61" t="n">
         <v>2</v>
       </c>
-      <c r="D59" t="n">
+      <c r="D61" t="n">
         <v>15.81</v>
       </c>
     </row>

</xml_diff>